<commit_message>
update check prompt, slide
</commit_message>
<xml_diff>
--- a/docx/Báo cáo/Test case kiểm thử chức năng.xlsx
+++ b/docx/Báo cáo/Test case kiểm thử chức năng.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnTotNghiep_NguyenQuyen_10122312\docx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnTotNghiep_NguyenQuyen_10122312\docx\Báo cáo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159DF095-C80B-413C-B9DE-F14ABA13DE48}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CB1A5C-CCB8-4156-B1FF-931F3E9D334E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9190" tabRatio="455" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9190" tabRatio="455" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TC_DangNhap" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="170">
   <si>
     <t>To Buglist</t>
   </si>
@@ -247,42 +247,10 @@
 Thông báo lỗi "Vui lòng điền vào trường này"</t>
   </si>
   <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: 
-B4: Nhập mật khẩu: ngminhtu
-B5: Nhập xác nhânh mật khẩu: ngminhtu
-B6: Nhấn "Đăng ký" </t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: ngminhtu@gmail.com
-B4: Nhập mật khẩu: 
-B5: Nhập xác nhânh mật khẩu: ngminhtu
-B6: Nhấn "Đăng ký" </t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: ngminhtu@gmail.com
-B4: Nhập mật khẩu: ngminhtu
-B5: Nhập xác nhânh mật khẩu: 
-B6: Nhấn "Đăng ký" </t>
-  </si>
-  <si>
     <t>bỏ trống xác nhận mật khẩu</t>
   </si>
   <si>
     <t>email thiếu @</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: ngminhtu.com
-B4: Nhập mật khẩu: ngminhtu
-B5: Nhập xác nhânh mật khẩu: ngminhtu
-B6: Nhấn "Đăng ký" </t>
   </si>
   <si>
     <t>Hiển thị trang chủ Ella
@@ -293,23 +261,7 @@
     <t>email thiếu sau @</t>
   </si>
   <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: ngminhtu@
-B4: Nhập mật khẩu: ngminhtu
-B5: Nhập xác nhânh mật khẩu: ngminhtu
-B6: Nhấn "Đăng ký" </t>
-  </si>
-  <si>
     <t>Mật khẩu &lt; 6 ký tự</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: ngminhtu@gmail.com
-B4: Nhập mật khẩu: ngmi
-B5: Nhập xác nhânh mật khẩu: ngmi
-B6: Nhấn "Đăng ký" </t>
   </si>
   <si>
     <t>Hiển thị trang chủ Ella
@@ -537,31 +489,7 @@
     <t>email thiếu trước @</t>
   </si>
   <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: @gmail.com
-B4: Nhập mật khẩu: ngminhtu
-B5: Nhập xác nhânh mật khẩu: ngminhtu
-B6: Nhấn "Đăng ký" </t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: hoanganh@gmail.com
-B4: Nhập mật khẩu: hoanganh
-B5: Nhập xác nhânh mật khẩu: hoanganh1
-B6: Nhấn "Đăng ký" </t>
-  </si>
-  <si>
     <t>vị trí dấu '.' sai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1: Truy cập vào website https://debac.vn/
-B2: Chọn chức năng đăng ký
-B3: Nhập email: ngminhtu@gmail.
-B4: Nhập mật khẩu: ngminhtu
-B5: Nhập xác nhânh mật khẩu: ngminhtu
-B6: Nhấn "Đăng ký" </t>
   </si>
   <si>
     <t>Hiển thị trang chủ Ella
@@ -970,6 +898,81 @@
   <si>
     <t>Đăng nhập thành công
 Hệ thống thông báo "Vui lòng nhập ít nhất một số điện thoại bạn đang sử dụng"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: ngminhtu@gmail.com
+B4: Nhập mật khẩu: ngmi
+B5: Nhập xác nhânh mật khẩu: ngmi
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: hoanganh@gmail.com
+B4: Nhập mật khẩu: hoanganh
+B5: Nhập xác nhânh mật khẩu: hoanganh1
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: 
+B4: Nhập mật khẩu: ngminhtu
+B5: Nhập xác nhânh mật khẩu: ngminhtu
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: ngminhtu@gmail.com
+B4: Nhập mật khẩu: 
+B5: Nhập xác nhânh mật khẩu: ngminhtu
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: ngminhtu@gmail.com
+B4: Nhập mật khẩu: ngminhtu
+B5: Nhập xác nhânh mật khẩu: 
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: ngminhtu.com
+B4: Nhập mật khẩu: ngminhtu
+B5: Nhập xác nhânh mật khẩu: ngminhtu
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: ngminhtu@
+B4: Nhập mật khẩu: ngminhtu
+B5: Nhập xác nhânh mật khẩu: ngminhtu
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: @gmail.com
+B4: Nhập mật khẩu: ngminhtu
+B5: Nhập xác nhânh mật khẩu: ngminhtu
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1: Truy cập vào website https://ella.vn/
+B2: Chọn chức năng đăng ký
+B3: Nhập email: ngminhtu@gmail.
+B4: Nhập mật khẩu: ngminhtu
+B5: Nhập xác nhânh mật khẩu: ngminhtu
+B6: Nhấn "Đăng ký" </t>
+  </si>
+  <si>
+    <t>Fail: 0</t>
   </si>
 </sst>
 </file>
@@ -2053,19 +2056,19 @@
         <v>[DangKy - 02]</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>63</v>
+        <v>160</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G6" s="19" t="s">
         <v>11</v>
@@ -2081,19 +2084,19 @@
         <v>[DangKy - 03]</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C7" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>104</v>
+        <v>161</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>12</v>
@@ -2102,7 +2105,7 @@
         <v>20</v>
       </c>
       <c r="I7" s="38" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="60">
@@ -2117,7 +2120,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>53</v>
+        <v>162</v>
       </c>
       <c r="E8" s="19" t="s">
         <v>52</v>
@@ -2145,7 +2148,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>54</v>
+        <v>163</v>
       </c>
       <c r="E9" s="19" t="s">
         <v>52</v>
@@ -2167,13 +2170,13 @@
         <v>[DangKy - 07]</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C10" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>55</v>
+        <v>164</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>52</v>
@@ -2195,19 +2198,19 @@
         <v>[DangKy - 06]</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C11" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>58</v>
+        <v>165</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G11" s="19" t="s">
         <v>11</v>
@@ -2223,19 +2226,19 @@
         <v>[DangKy - 08]</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C12" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>61</v>
+        <v>166</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G12" s="19" t="s">
         <v>11</v>
@@ -2251,19 +2254,19 @@
         <v>[DangKy - 09]</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C13" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>103</v>
+        <v>167</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G13" s="19" t="s">
         <v>11</v>
@@ -2279,19 +2282,19 @@
         <v>[DangKy - 10]</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C14" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>106</v>
+        <v>168</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="G14" s="19" t="s">
         <v>11</v>
@@ -2395,7 +2398,7 @@
         <v>15</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>16</v>
+        <v>169</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>17</v>
@@ -2425,13 +2428,13 @@
         <v>9</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="G5" s="19" t="s">
         <v>11</v>
@@ -2446,19 +2449,19 @@
         <v>[TimKiemSP - 02]</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G6" s="19" t="s">
         <v>11</v>
@@ -2473,19 +2476,19 @@
         <v>[TimKiemSP - 03]</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C7" s="31" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="G7" s="19" t="s">
         <v>11</v>
@@ -2507,13 +2510,13 @@
         <v>9</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>11</v>
@@ -2529,19 +2532,19 @@
         <v>[TimKiemSP - 05]</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="G9" s="28" t="s">
         <v>11</v>
@@ -2557,19 +2560,19 @@
         <v>[TimKiemSP - 06]</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C10" s="31" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G10" s="28" t="s">
         <v>11</v>
@@ -2620,10 +2623,10 @@
   <sheetData>
     <row r="4" spans="6:9" ht="14.5">
       <c r="F4" s="40" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="G4" s="40" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="H4" s="40" t="s">
         <v>11</v>
@@ -2634,7 +2637,7 @@
     </row>
     <row r="5" spans="6:9" ht="14.5">
       <c r="F5" s="39" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="G5" s="41">
         <v>10</v>
@@ -2648,7 +2651,7 @@
     </row>
     <row r="6" spans="6:9" ht="14.5">
       <c r="F6" s="45" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="G6" s="46">
         <v>5</v>
@@ -2662,7 +2665,7 @@
     </row>
     <row r="7" spans="6:9" ht="14.5">
       <c r="F7" s="39" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="G7" s="41">
         <v>6</v>
@@ -2676,7 +2679,7 @@
     </row>
     <row r="8" spans="6:9" ht="14.5">
       <c r="F8" s="45" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="G8" s="46">
         <v>11</v>
@@ -2690,7 +2693,7 @@
     </row>
     <row r="9" spans="6:9" ht="14.5">
       <c r="F9" s="39" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="G9" s="41">
         <v>11</v>
@@ -2704,7 +2707,7 @@
     </row>
     <row r="10" spans="6:9" ht="14.5">
       <c r="F10" s="45" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="G10" s="46">
         <v>8</v>
@@ -2718,7 +2721,7 @@
     </row>
     <row r="11" spans="6:9" ht="14.5">
       <c r="F11" s="43" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="G11" s="44">
         <f>SUM(G5:G10)</f>
@@ -2855,13 +2858,13 @@
         <v>10</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="G5" s="19" t="s">
         <v>11</v>
@@ -2877,19 +2880,19 @@
         <v>[ThanhToan - 02]</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="G6" s="19" t="s">
         <v>11</v>
@@ -2905,19 +2908,19 @@
         <v>[ThanhToan - 03]</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C7" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>12</v>
@@ -2926,7 +2929,7 @@
         <v>20</v>
       </c>
       <c r="I7" s="38" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="100">
@@ -2935,19 +2938,19 @@
         <v>[ThanhToan - 04]</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="C8" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>11</v>
@@ -2963,19 +2966,19 @@
         <v>[ThanhToan - 05]</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>11</v>
@@ -2997,13 +3000,13 @@
         <v>10</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G10" s="19" t="s">
         <v>11</v>
@@ -3025,13 +3028,13 @@
         <v>10</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G11" s="19" t="s">
         <v>11</v>
@@ -3047,19 +3050,19 @@
         <v>[ThanhToan - 08]</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="C12" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="G12" s="19" t="s">
         <v>11</v>
@@ -3075,19 +3078,19 @@
         <v>[ThanhToan - 09]</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="C13" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="G13" s="19" t="s">
         <v>11</v>
@@ -3103,19 +3106,19 @@
         <v>[ThanhToan - 10]</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C14" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="G14" s="19" t="s">
         <v>11</v>
@@ -3131,19 +3134,19 @@
         <v>[ThanhToan - 11]</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C15" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="G15" s="19" t="s">
         <v>11</v>
@@ -3273,19 +3276,19 @@
         <v>[ChangeProfile - 01]</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C5" s="31" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G5" s="19" t="s">
         <v>11</v>
@@ -3307,13 +3310,13 @@
         <v>13</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G6" s="19" t="s">
         <v>11</v>
@@ -3335,13 +3338,13 @@
         <v>13</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G7" s="19" t="s">
         <v>11</v>
@@ -3357,19 +3360,19 @@
         <v>[ChangeProfile - 04]</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C8" s="31" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>11</v>
@@ -3385,19 +3388,19 @@
         <v>[ChangeProfile - 05]</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>12</v>
@@ -3406,7 +3409,7 @@
         <v>20</v>
       </c>
       <c r="I9" s="38" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="80">
@@ -3415,19 +3418,19 @@
         <v>[ChangeProfile - 06]</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C10" s="31" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>12</v>
@@ -3436,7 +3439,7 @@
         <v>20</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="80">
@@ -3445,19 +3448,19 @@
         <v>[ChangeProfile - 07]</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="C11" s="31" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>12</v>
@@ -3466,7 +3469,7 @@
         <v>20</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="80">
@@ -3475,19 +3478,19 @@
         <v>[ChangeProfile - 08]</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C12" s="31" t="s">
         <v>13</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>12</v>
@@ -3496,20 +3499,21 @@
         <v>20</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B1" location="BugList!A1" display="To Buglist" xr:uid="{6F980733-6528-424B-B45A-75D8EB680571}"/>
     <hyperlink ref="A1" r:id="rId1" xr:uid="{79014417-D33A-48E5-ABCD-22679886FC3B}"/>
-    <hyperlink ref="I9" r:id="rId2" display="..\screenshots\E2E_login_20260517_213426_5_20260519_030532.png" xr:uid="{24F2C39C-A2BF-4E1D-BEC4-DB37E8FBD3D9}"/>
+    <hyperlink ref="I9" r:id="rId2" xr:uid="{24F2C39C-A2BF-4E1D-BEC4-DB37E8FBD3D9}"/>
     <hyperlink ref="I10" r:id="rId3" xr:uid="{E5BA72D2-91F9-470C-A182-B694505EAA04}"/>
     <hyperlink ref="I11" r:id="rId4" xr:uid="{AE3A4F13-1BDE-4CB0-852A-ED458A6944D6}"/>
     <hyperlink ref="I12" r:id="rId5" xr:uid="{B9092595-C182-4014-8309-32004122821E}"/>
     <hyperlink ref="I9:I12" r:id="rId6" display="E2E_login_20260517_213426_5_.png" xr:uid="{AA14C026-3BC7-4CAE-A88E-E9CEB146D70C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 
@@ -3628,13 +3632,13 @@
         <v>10</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G5" s="19" t="s">
         <v>11</v>
@@ -3650,19 +3654,19 @@
         <v>[ThanhToan - 02]</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="G6" s="19" t="s">
         <v>11</v>
@@ -3678,19 +3682,19 @@
         <v>[ThanhToan - 03]</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C7" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>12</v>
@@ -3699,7 +3703,7 @@
         <v>20</v>
       </c>
       <c r="I7" s="38" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="120">
@@ -3708,19 +3712,19 @@
         <v>[ThanhToan - 04]</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="C8" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>11</v>
@@ -3736,19 +3740,19 @@
         <v>[ThanhToan - 05]</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>11</v>
@@ -3770,13 +3774,13 @@
         <v>10</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="G10" s="19" t="s">
         <v>11</v>
@@ -3798,13 +3802,13 @@
         <v>10</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="G11" s="19" t="s">
         <v>11</v>
@@ -3820,19 +3824,19 @@
         <v>[ThanhToan - 07]</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="C12" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="G12" s="19" t="s">
         <v>11</v>
@@ -3848,19 +3852,19 @@
         <v>[ThanhToan - 08]</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="C13" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="G13" s="19" t="s">
         <v>11</v>
@@ -3876,19 +3880,19 @@
         <v>[ThanhToan - 10]</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C14" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="G14" s="19" t="s">
         <v>11</v>
@@ -3904,19 +3908,19 @@
         <v>[ThanhToan - 11]</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C15" s="31" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="G15" s="19" t="s">
         <v>11</v>

</xml_diff>